<commit_message>
Create Pasta de projeto CAD
</commit_message>
<xml_diff>
--- a/Montagem, Instalação e Integração de Sistemas Robóticos/PE Montagem, Instalação e Integração de Sistemas Robóticos FRC.xlsx
+++ b/Montagem, Instalação e Integração de Sistemas Robóticos/PE Montagem, Instalação e Integração de Sistemas Robóticos FRC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djair.oliveira\Documents\GitHub\Curso 2026\Montagem, Instalação e Integração de Sistemas Robóticos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D8411B2-D093-4229-A973-724765F2C533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58B892BC-561A-431B-9A51-F6AA82299389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLANO DE ENSINO" sheetId="3" r:id="rId1"/>
@@ -56,7 +56,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Segoe UI"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Preencher com o nome da unidade operacional, responsável pelo curso.</t>
         </r>
@@ -666,12 +666,6 @@
     <t>20 Horas</t>
   </si>
   <si>
-    <t>50 Horas</t>
-  </si>
-  <si>
-    <t>18 Horas</t>
-  </si>
-  <si>
     <t>1 Horas</t>
   </si>
   <si>
@@ -710,12 +704,18 @@
 • Registrar observações importantes no Engineering Notebook.
 • Reportar status do progresso aos mentores e colegas.</t>
   </si>
+  <si>
+    <t>16 Horas</t>
+  </si>
+  <si>
+    <t>56 Horas</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -729,12 +729,6 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Segoe UI"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
@@ -1028,74 +1022,74 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -1108,14 +1102,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1123,84 +1114,87 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1908,10 +1902,10 @@
     </row>
     <row r="17" spans="2:8" ht="93" customHeight="1">
       <c r="B17" s="3" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>63</v>
@@ -1931,10 +1925,10 @@
     </row>
     <row r="18" spans="2:8" ht="150">
       <c r="B18" s="3" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D18" s="21" t="s">
         <v>64</v>
@@ -1957,7 +1951,7 @@
         <v>71</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D19" s="21" t="s">
         <v>65</v>
@@ -1977,10 +1971,10 @@
     </row>
     <row r="20" spans="2:8" ht="270">
       <c r="B20" s="3" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D20" s="21" t="s">
         <v>66</v>
@@ -2003,7 +1997,7 @@
         <v>49</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D21" s="21" t="s">
         <v>67</v>
@@ -2026,7 +2020,7 @@
         <v>48</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>68</v>
@@ -2049,7 +2043,7 @@
         <v>50</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>69</v>
@@ -2069,10 +2063,10 @@
     </row>
     <row r="24" spans="2:8" ht="210">
       <c r="B24" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>70</v>
@@ -3412,22 +3406,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="900f5ea3-4309-4848-96c1-ad4c68ce6813">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06146d02-393f-48de-94b9-ef7e514a30fa" xsi:nil="true"/>
-    <_dlc_DocId xmlns="06146d02-393f-48de-94b9-ef7e514a30fa">ETSV6M6J7ZTN-240384884-35593</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="06146d02-393f-48de-94b9-ef7e514a30fa">
-      <Url>https://senaimt.sharepoint.com/sites/sfiemt/_layouts/15/DocIdRedir.aspx?ID=ETSV6M6J7ZTN-240384884-35593</Url>
-      <Description>ETSV6M6J7ZTN-240384884-35593</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -3477,7 +3455,7 @@
 </spe:Receivers>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -3486,7 +3464,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C644A9542FF24642A542429309CC4519" ma:contentTypeVersion="23" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="bc4dd412d0023e8c739373a37bde5358">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="900f5ea3-4309-4848-96c1-ad4c68ce6813" xmlns:ns3="06146d02-393f-48de-94b9-ef7e514a30fa" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d520e6f3725bd97d2cbca1e5ca693b32" ns2:_="" ns3:_="">
     <xsd:import namespace="900f5ea3-4309-4848-96c1-ad4c68ce6813"/>
@@ -3772,18 +3750,23 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA13BBC6-8A75-4AE6-9EEA-9BB889D14091}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="900f5ea3-4309-4848-96c1-ad4c68ce6813"/>
-    <ds:schemaRef ds:uri="06146d02-393f-48de-94b9-ef7e514a30fa"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="900f5ea3-4309-4848-96c1-ad4c68ce6813">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06146d02-393f-48de-94b9-ef7e514a30fa" xsi:nil="true"/>
+    <_dlc_DocId xmlns="06146d02-393f-48de-94b9-ef7e514a30fa">ETSV6M6J7ZTN-240384884-35593</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="06146d02-393f-48de-94b9-ef7e514a30fa">
+      <Url>https://senaimt.sharepoint.com/sites/sfiemt/_layouts/15/DocIdRedir.aspx?ID=ETSV6M6J7ZTN-240384884-35593</Url>
+      <Description>ETSV6M6J7ZTN-240384884-35593</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20786E8E-CB34-4DAA-8592-D1F9484BF044}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
@@ -3791,7 +3774,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81A6ECAD-A0AB-448D-840C-F95861E92F39}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -3799,7 +3782,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{34BF3B50-FE1F-4615-B748-8C7173D9647D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3816,4 +3799,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA13BBC6-8A75-4AE6-9EEA-9BB889D14091}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="900f5ea3-4309-4848-96c1-ad4c68ce6813"/>
+    <ds:schemaRef ds:uri="06146d02-393f-48de-94b9-ef7e514a30fa"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>